<commit_message>
chore: remove outdated simulation data for Crucible 1 and Crucible 2 shield configurations
</commit_message>
<xml_diff>
--- a/data/output/great.xlsx
+++ b/data/output/great.xlsx
@@ -52,60 +52,60 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Toxapex PJ+SW/Bri 0/15/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>fairy/none</t>
+          <t>poison/water</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Corviknight SdA+AC/Pbk 0/13/14</t>
+          <t>Talonflame I+BrB/Fl 0/13/14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flying/steel</t>
+          <t>fire/flying</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Tinkaton FW+PR/Bd 3/10/12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>water/ground</t>
+          <t>fairy/steel</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tinkaton FW+PR/Bd 3/10/12</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fairy/steel</t>
+          <t>ground/ghost</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Corsola (Galarian) A+PG/NSh 11/12/12</t>
+          <t>Lapras Psy+IB/SpA 0/10/14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ghost/none</t>
+          <t>water/ice</t>
         </is>
       </c>
     </row>
@@ -165,7 +165,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>208.68168893058365</v>
+        <v>211.95628592470962</v>
       </c>
     </row>
     <row r="6">
@@ -175,7 +175,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>813.8933333333333</v>
+        <v>867.68</v>
       </c>
     </row>
     <row r="7">
@@ -185,7 +185,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>23.0</v>
+        <v>-1.0</v>
       </c>
     </row>
     <row r="8">
@@ -195,7 +195,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9">
@@ -205,7 +205,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.8266666666666667</v>
+        <v>0.9333333333333333</v>
       </c>
     </row>
     <row r="10">
@@ -215,7 +215,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
@@ -225,7 +225,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">
@@ -235,7 +235,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>751.8933333333333</v>
+        <v>797.68</v>
       </c>
     </row>
     <row r="13">
@@ -255,7 +255,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>733.1199999999999</v>
+        <v>764.2213523809525</v>
       </c>
     </row>
     <row r="15">
@@ -265,7 +265,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>632.7109333333333</v>
+        <v>660.9762714285714</v>
       </c>
     </row>
     <row r="16">
@@ -275,7 +275,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>719.5173333333333</v>
+        <v>755.1916571428571</v>
       </c>
     </row>
     <row r="17">
@@ -295,7 +295,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>751.8933333333333</v>
+        <v>797.68</v>
       </c>
     </row>
     <row r="19">
@@ -305,7 +305,7 @@
         </is>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -315,7 +315,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>0.02</v>
+        <v>0.006666666666666667</v>
       </c>
     </row>
     <row r="21">
@@ -325,7 +325,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>27.20000000000001</v>
+        <v>28.80000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -355,149 +355,159 @@
         </is>
       </c>
       <c r="B24">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>redundant_coverage_2plus</t>
+          <t>ranking_aware_score</t>
         </is>
       </c>
       <c r="B25">
-        <v>136</v>
+        <v>0.7252973698039533</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>redundant_coverage_3plus</t>
+          <t>redundant_coverage_2plus</t>
         </is>
       </c>
       <c r="B26">
-        <v>103</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>safe_member_floor</t>
+          <t>redundant_coverage_3plus</t>
         </is>
       </c>
       <c r="B27">
-        <v>90.0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>safe_member_target</t>
+          <t>safe_member_floor</t>
         </is>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>90.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>safety_floor_target</t>
+          <t>safe_member_target</t>
         </is>
       </c>
       <c r="B29">
-        <v>78.0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>safety_pool_max</t>
+          <t>safety_floor_target</t>
         </is>
       </c>
       <c r="B30">
-        <v>95.6</v>
+        <v>78.0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>safety_pool_mean</t>
+          <t>safety_pool_max</t>
         </is>
       </c>
       <c r="B31">
-        <v>76.032</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>safety_pool_min</t>
+          <t>safety_pool_mean</t>
         </is>
       </c>
       <c r="B32">
-        <v>45.6</v>
+        <v>77.452</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>safety_priority</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+          <t>safety_pool_min</t>
+        </is>
+      </c>
+      <c r="B33">
+        <v>41.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>safety_score</t>
-        </is>
-      </c>
-      <c r="B34">
-        <v>80.11666666666666</v>
+          <t>safety_priority</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>single_cover_pairs</t>
+          <t>safety_score</t>
         </is>
       </c>
       <c r="B35">
-        <v>11</v>
+        <v>79.18333333333334</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>single_cover_rate</t>
+          <t>single_cover_pairs</t>
         </is>
       </c>
       <c r="B36">
-        <v>0.07333333333333333</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>total_pairs</t>
+          <t>single_cover_rate</t>
         </is>
       </c>
       <c r="B37">
-        <v>150</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>total_pairs</t>
+        </is>
+      </c>
+      <c r="B38">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>weighted_worst_best_score</t>
         </is>
       </c>
-      <c r="B38">
-        <v>682.9999999999999</v>
+      <c r="B39">
+        <v>730.8571428571431</v>
       </c>
     </row>
   </sheetData>
@@ -556,16 +566,16 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0.959184</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -651,97 +661,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gourgeist (Large) I+SB/SeB 1/14/15</t>
+          <t>Gastrodon MSl+BS/WP 1/15/14</t>
         </is>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1-shield no cover</t>
+          <t>0-shield only Lapras Psy+IB/SpA 0/10/14 | 2-shield no cover</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Talonflame (Shadow) I+FmC/Fl 0/13/15</t>
+          <t>Stunfisk TS+MB/D 0/12/15</t>
         </is>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2-shield no cover</t>
+          <t>1-shield only Golurk (Shadow) MSl+DyP/ShP 0/12/11 | 2-shield only Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cradily Ac+RT/GK 0/15/15</t>
+          <t>Jellicent H+S/SB 1/14/14</t>
         </is>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1-shield no cover</t>
+          <t>0-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15 | 2-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ludicolo A+WBW/LfS 0/15/15</t>
+          <t>Lickilicky RO+BS/SB 0/15/10</t>
         </is>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0-shield only Corviknight SdA+AC/Pbk 0/13/14 | 1-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
+          <t>2-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+BS/WP 1/15/14</t>
+          <t>Dusknoir (Shadow) A+DyP/ShP 0/14/13</t>
         </is>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0-shield only Corsola (Galarian) A+PG/NSh 11/12/12 | 2-shield only Corviknight SdA+AC/Pbk 0/13/14</t>
+          <t>2-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Azumarill B+IB/PR 0/15/15</t>
+          <t>Primeape KC+RF/CC 1/15/15</t>
         </is>
       </c>
       <c r="B7">
@@ -752,14 +762,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0-shield only Tinkaton FW+PR/Bd 3/10/12</t>
+          <t>2-shield only Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Primeape KC+RF/CC 1/15/15</t>
+          <t>Charjabug VS+XS/D 0/13/15</t>
         </is>
       </c>
       <c r="B8">
@@ -770,14 +780,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2-shield only Clefable FW+M/MM 2/12/11</t>
+          <t>1-shield only Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Stunfisk TS+MB/D 0/12/15</t>
+          <t>Steelix TF+PsF/Cr 0/14/15</t>
         </is>
       </c>
       <c r="B9">
@@ -788,14 +798,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2-shield only Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>2-shield only Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Steelix TF+PsF/Cr 0/14/15</t>
+          <t>Empoleon (Shadow) MSo+HC/DrlP 0/13/15</t>
         </is>
       </c>
       <c r="B10">
@@ -806,14 +816,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2-shield only Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>0-shield only Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Clodsire PSt+Eq/SE 0/14/13</t>
+          <t>Guzzlord DT+BrS/SlB 1/15/15</t>
         </is>
       </c>
       <c r="B11">
@@ -824,7 +834,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0-shield only Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>2-shield only Tinkaton FW+PR/Bd 3/10/12</t>
         </is>
       </c>
     </row>
@@ -888,17 +898,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
+          <t>Talonflame I+BrB/Fl 0/13/14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -907,16 +917,16 @@
         </is>
       </c>
       <c r="F2">
-        <v>733.1199999999999</v>
+        <v>764.7687282633902</v>
       </c>
       <c r="G2">
-        <v>733.1199999999999</v>
+        <v>747.9466666666667</v>
       </c>
       <c r="H2">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -930,12 +940,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Talonflame I+BrB/Fl 0/13/14</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -944,16 +954,16 @@
         </is>
       </c>
       <c r="F3">
-        <v>732.2466666666666</v>
+        <v>762.6754607892517</v>
       </c>
       <c r="G3">
-        <v>732.2466666666666</v>
+        <v>744.8066666666667</v>
       </c>
       <c r="H3">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -962,12 +972,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Talonflame I+BrB/Fl 0/13/14</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -981,16 +991,16 @@
         </is>
       </c>
       <c r="F4">
-        <v>731.6266666666667</v>
+        <v>759.7567284573835</v>
       </c>
       <c r="G4">
-        <v>731.6266666666667</v>
+        <v>742.48</v>
       </c>
       <c r="H4">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -999,17 +1009,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tinkaton FW+PR/Bd 3/10/12</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
+          <t>Toxapex PJ+SW/Bri 0/15/15</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1018,13 +1028,13 @@
         </is>
       </c>
       <c r="F5">
-        <v>718.96</v>
+        <v>758.3216025154621</v>
       </c>
       <c r="G5">
-        <v>718.96</v>
+        <v>740.32</v>
       </c>
       <c r="H5">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -1041,12 +1051,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tinkaton FW+PR/Bd 3/10/12</t>
+          <t>Toxapex PJ+SW/Bri 0/15/15</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1055,16 +1065,16 @@
         </is>
       </c>
       <c r="F6">
-        <v>718.8266666666667</v>
+        <v>758.1423350413237</v>
       </c>
       <c r="G6">
-        <v>718.8266666666667</v>
+        <v>739.3066666666667</v>
       </c>
       <c r="H6">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1073,17 +1083,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gastrodon MSl+WP/BS 1/15/14</t>
+          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tinkaton FW+PR/Bd 3/10/12</t>
+          <t>Lapras Psy+IB/SpA 0/10/14</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1092,16 +1102,16 @@
         </is>
       </c>
       <c r="F7">
-        <v>716.3866666666667</v>
+        <v>754.7345923543503</v>
       </c>
       <c r="G7">
-        <v>716.3866666666667</v>
+        <v>734.9133333333333</v>
       </c>
       <c r="H7">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1110,12 +1120,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Corviknight SdA+AC/Pbk 0/13/14</t>
+          <t>Toxapex PJ+SW/Bri 0/15/15</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1129,16 +1139,16 @@
         </is>
       </c>
       <c r="F8">
-        <v>713.84</v>
+        <v>754.5403603377523</v>
       </c>
       <c r="G8">
-        <v>713.84</v>
+        <v>736.7133333333333</v>
       </c>
       <c r="H8">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1147,35 +1157,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Lapras Psy+IB/SpA 0/10/14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Corviknight SdA+AC/Pbk 0/13/14</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
       <c r="F9">
-        <v>712.4266666666667</v>
+        <v>752.7953849426946</v>
       </c>
       <c r="G9">
-        <v>712.4266666666667</v>
+        <v>734.0333333333333</v>
       </c>
       <c r="H9">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1184,17 +1194,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Corviknight SdA+AC/Pbk 0/13/14</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Morpeko (Full Belly) TS+AuW/PsF 10/12/15</t>
+          <t>Tinkaton FW+PR/Bd 3/10/12</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1203,16 +1213,16 @@
         </is>
       </c>
       <c r="F10">
-        <v>712.3333333333334</v>
+        <v>752.4765076255438</v>
       </c>
       <c r="G10">
-        <v>712.3333333333334</v>
+        <v>732.66</v>
       </c>
       <c r="H10">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1221,12 +1231,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Corsola (Galarian) A+PG/NSh 11/12/12</t>
+          <t>Tinkaton FW+PR/Bd 3/10/12</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Clefable FW+M/MM 2/12/11</t>
+          <t>Golurk (Shadow) MSl+DyP/ShP 0/12/11</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1236,20 +1246,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ABA</t>
+          <t>ABC</t>
         </is>
       </c>
       <c r="F11">
-        <v>705.4066666666666</v>
+        <v>751.6122337071448</v>
       </c>
       <c r="G11">
-        <v>705.4066666666666</v>
+        <v>731.7533333333334</v>
       </c>
       <c r="H11">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1312,13 +1322,13 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>746.76</v>
+        <v>754.76</v>
       </c>
       <c r="F2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1337,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>745.92</v>
+        <v>778.9</v>
       </c>
       <c r="F3">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1362,10 +1372,10 @@
         <v>2</v>
       </c>
       <c r="E4">
-        <v>706.68</v>
+        <v>710.18</v>
       </c>
       <c r="F4">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1387,13 +1397,13 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>746.76</v>
+        <v>754.76</v>
       </c>
       <c r="F5">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1412,10 +1422,10 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>707.98</v>
+        <v>721.12</v>
       </c>
       <c r="F6">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1437,7 +1447,7 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>742.0</v>
+        <v>758.54</v>
       </c>
       <c r="F7">
         <v>40</v>
@@ -1462,13 +1472,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>746.76</v>
+        <v>754.76</v>
       </c>
       <c r="F8">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1487,10 +1497,10 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>740.46</v>
+        <v>727.88</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1512,10 +1522,10 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>707.66</v>
+        <v>744.8</v>
       </c>
       <c r="F10">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1537,13 +1547,13 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>729.26</v>
+        <v>758.38</v>
       </c>
       <c r="F11">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1562,13 +1572,13 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>730.18</v>
+        <v>762.54</v>
       </c>
       <c r="F12">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1587,13 +1597,13 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>697.44</v>
+        <v>700.04</v>
       </c>
       <c r="F13">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1612,13 +1622,13 @@
         <v>1</v>
       </c>
       <c r="E14">
-        <v>729.26</v>
+        <v>758.38</v>
       </c>
       <c r="F14">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1637,13 +1647,13 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>695.1</v>
+        <v>718.28</v>
       </c>
       <c r="F15">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1662,13 +1672,13 @@
         <v>2</v>
       </c>
       <c r="E16">
-        <v>732.12</v>
+        <v>741.26</v>
       </c>
       <c r="F16">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1687,13 +1697,13 @@
         <v>1</v>
       </c>
       <c r="E17">
-        <v>729.26</v>
+        <v>745.68</v>
       </c>
       <c r="F17">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1712,10 +1722,10 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>735.38</v>
+        <v>712.1</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -1737,13 +1747,13 @@
         <v>2</v>
       </c>
       <c r="E19">
-        <v>684.52</v>
+        <v>746.96</v>
       </c>
       <c r="F19">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1762,10 +1772,10 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>719.44</v>
+        <v>758.38</v>
       </c>
       <c r="F20">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1787,13 +1797,13 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>748.16</v>
+        <v>720.98</v>
       </c>
       <c r="F21">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1812,13 +1822,13 @@
         <v>2</v>
       </c>
       <c r="E22">
-        <v>673.92</v>
+        <v>730.78</v>
       </c>
       <c r="F22">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -1837,7 +1847,7 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>719.44</v>
+        <v>745.68</v>
       </c>
       <c r="F23">
         <v>44</v>
@@ -1862,10 +1872,10 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>683.34</v>
+        <v>725.26</v>
       </c>
       <c r="F24">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -1887,13 +1897,13 @@
         <v>2</v>
       </c>
       <c r="E25">
-        <v>734.5</v>
+        <v>731.16</v>
       </c>
       <c r="F25">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1912,13 +1922,13 @@
         <v>1</v>
       </c>
       <c r="E26">
-        <v>719.44</v>
+        <v>751.9</v>
       </c>
       <c r="F26">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1937,13 +1947,13 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>717.88</v>
+        <v>693.02</v>
       </c>
       <c r="F27">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1962,13 +1972,13 @@
         <v>2</v>
       </c>
       <c r="E28">
-        <v>699.68</v>
+        <v>753.06</v>
       </c>
       <c r="F28">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -1987,10 +1997,10 @@
         <v>1</v>
       </c>
       <c r="E29">
-        <v>710.04</v>
+        <v>751.9</v>
       </c>
       <c r="F29">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -2012,10 +2022,10 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>717.78</v>
+        <v>734.12</v>
       </c>
       <c r="F30">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="G30">
         <v>0</v>
@@ -2037,13 +2047,13 @@
         <v>2</v>
       </c>
       <c r="E31">
-        <v>688.4</v>
+        <v>709.24</v>
       </c>
       <c r="F31">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>